<commit_message>
Refactor self vs partner report correlations and update data prep
Moved self vs partner report correlation analysis from 00_Descriptives.Rmd to 01_MainModels.Rmd and updated the variables used to match new naming conventions. Added relevant variables to the data selection in PrepareData.R to ensure they are available for analysis. Updated output Excel files to reflect these changes.
</commit_message>
<xml_diff>
--- a/Output/DescriptivesAll.xlsx
+++ b/Output/DescriptivesAll.xlsx
@@ -1,212 +1,205 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pascku\Repos\02TimeAndTiesControl\Output\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50C10368-58A4-499D-918B-316DF6B69820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="-22510" yWindow="760" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
-  <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>Level</t>
-  </si>
-  <si>
-    <t>n Observations</t>
-  </si>
-  <si>
-    <t>% Observations</t>
-  </si>
-  <si>
-    <t>Missing</t>
-  </si>
-  <si>
-    <t>Mean</t>
-  </si>
-  <si>
-    <t>SD</t>
-  </si>
-  <si>
-    <t>Range</t>
-  </si>
-  <si>
-    <t>persuasion</t>
-  </si>
-  <si>
-    <t>6%</t>
-  </si>
-  <si>
-    <t>0.00-   5.00</t>
-  </si>
-  <si>
-    <t>pressure</t>
-  </si>
-  <si>
-    <t>pushing</t>
-  </si>
-  <si>
-    <t>7%</t>
-  </si>
-  <si>
-    <t>pa_sub</t>
-  </si>
-  <si>
-    <t>0.00- 720.00</t>
-  </si>
-  <si>
-    <t>pa_obj</t>
-  </si>
-  <si>
-    <t>11%</t>
-  </si>
-  <si>
-    <t>5.75- 971.25</t>
-  </si>
-  <si>
-    <t>aff</t>
-  </si>
-  <si>
-    <t>reactance</t>
-  </si>
-  <si>
-    <t>81%</t>
-  </si>
-  <si>
-    <t>day</t>
-  </si>
-  <si>
-    <t>0%</t>
-  </si>
-  <si>
-    <t>0.00-   1.00</t>
-  </si>
-  <si>
-    <t>weartime</t>
-  </si>
-  <si>
-    <t>1%</t>
-  </si>
-  <si>
-    <t>0.00-1440.00</t>
-  </si>
-  <si>
-    <t>isWeekend</t>
-  </si>
-  <si>
-    <t>Weekend</t>
-  </si>
-  <si>
-    <t>29%</t>
-  </si>
-  <si>
-    <t>Weekday</t>
-  </si>
-  <si>
-    <t>71%</t>
-  </si>
-  <si>
-    <t>barriers</t>
-  </si>
-  <si>
-    <t>56%</t>
-  </si>
-  <si>
-    <t>0.00-   3.50</t>
-  </si>
-  <si>
-    <t>facilitators</t>
-  </si>
-  <si>
-    <t>plan</t>
-  </si>
-  <si>
-    <t>missing</t>
-  </si>
-  <si>
-    <t>Plan</t>
-  </si>
-  <si>
-    <t>44%</t>
-  </si>
-  <si>
-    <t>No plan</t>
-  </si>
-  <si>
-    <t>49%</t>
-  </si>
-  <si>
-    <t>studyGroup</t>
-  </si>
-  <si>
-    <t>last 3 weeks interventions</t>
-  </si>
-  <si>
-    <t>32%</t>
-  </si>
-  <si>
-    <t>Allways inerventions</t>
-  </si>
-  <si>
-    <t>34%</t>
-  </si>
-  <si>
-    <t>First 3 weeks interventions</t>
-  </si>
-  <si>
-    <t>support</t>
-  </si>
-  <si>
-    <t>got_JITAI</t>
-  </si>
-  <si>
-    <t>JITAI received</t>
-  </si>
-  <si>
-    <t>14%</t>
-  </si>
-  <si>
-    <t>No JITAI</t>
-  </si>
-  <si>
-    <t>86%</t>
-  </si>
-  <si>
-    <t>skilled_support</t>
-  </si>
-  <si>
-    <t>Days before Intervention</t>
-  </si>
-  <si>
-    <t>25%</t>
-  </si>
-  <si>
-    <t>Days after Intervention</t>
-  </si>
-  <si>
-    <t>75%</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+  <si>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n Observations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% Observations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">persuasion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00-   5.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pushing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pa_sub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00- 720.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pa_obj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.75- 971.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reactance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00-   1.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weartime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00-1440.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">isWeekend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">71%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barriers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">56%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00-   3.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">facilitators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">missing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">studyGroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last 3 weeks interventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allways inerventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First 3 weeks interventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">support</t>
+  </si>
+  <si>
+    <t xml:space="preserve">got_JITAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JITAI received</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No JITAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">skilled_support</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days before Intervention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days after Intervention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -237,28 +230,20 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -268,23 +253,11 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -566,21 +539,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.46484375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.9296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.265625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -606,212 +569,212 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="2">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="2">
+      <c r="C2" s="2" t="n">
         <v>3936</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="2" t="n">
         <v>0.42</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="2" t="n">
         <v>1.08</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="1">
+      <c r="C3" s="1" t="n">
         <v>3931</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="1" t="n">
         <v>0.12</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="1" t="n">
         <v>0.62</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="1">
+      <c r="C4" s="1" t="n">
         <v>3905</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="1" t="n">
         <v>0.16</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="1" t="n">
         <v>0.66</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="5">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="1"/>
-      <c r="C5" s="1">
+      <c r="C5" s="1" t="n">
         <v>3943</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="1" t="n">
         <v>30.4</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="1" t="n">
         <v>54.78</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6">
       <c r="A6" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="1"/>
-      <c r="C6" s="1">
+      <c r="C6" s="1" t="n">
         <v>3706</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="1" t="n">
         <v>144.41</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="1" t="n">
         <v>117.81</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7">
       <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="1"/>
-      <c r="C7" s="1">
+      <c r="C7" s="1" t="n">
         <v>3944</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="1" t="n">
         <v>3.83</v>
       </c>
-      <c r="G7" s="1">
-        <v>1.1399999999999999</v>
+      <c r="G7" s="1" t="n">
+        <v>1.14</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8">
       <c r="A8" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="1"/>
-      <c r="C8" s="1">
+      <c r="C8" s="1" t="n">
         <v>795</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="1" t="n">
         <v>0.79</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="1" t="n">
         <v>1.32</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="9">
       <c r="A9" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="1"/>
-      <c r="C9" s="1">
+      <c r="C9" s="1" t="n">
         <v>4180</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="G9" s="1">
-        <v>0.28999999999999998</v>
+      <c r="G9" s="1" t="n">
+        <v>0.29</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="10">
       <c r="A10" t="s">
         <v>25</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="C10" s="1">
+      <c r="C10" s="1" t="n">
         <v>4124</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="1" t="n">
         <v>1057.42</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="1" t="n">
         <v>384.29</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="11">
       <c r="A11" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="1" t="n">
         <v>1216</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -822,14 +785,14 @@
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="12">
       <c r="A12" t="s">
         <v>28</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="1" t="n">
         <v>2964</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -840,58 +803,58 @@
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="13">
       <c r="A13" t="s">
         <v>33</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="1">
+      <c r="C13" s="1" t="n">
         <v>1856</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="1" t="n">
         <v>0.9</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="1" t="n">
         <v>0.75</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="14">
       <c r="A14" t="s">
         <v>36</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="1">
+      <c r="C14" s="1" t="n">
         <v>1856</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="1" t="n">
         <v>0.92</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="1" t="n">
         <v>1.02</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="15">
       <c r="A15" t="s">
         <v>37</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="1" t="n">
         <v>272</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -902,14 +865,14 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="16">
       <c r="A16" t="s">
         <v>37</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="1" t="n">
         <v>1860</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -920,14 +883,14 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="17">
       <c r="A17" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="1" t="n">
         <v>2048</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -938,14 +901,14 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="18">
       <c r="A18" t="s">
         <v>43</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="1" t="n">
         <v>1320</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -956,14 +919,14 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="19">
       <c r="A19" t="s">
         <v>43</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="1" t="n">
         <v>1430</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -974,14 +937,14 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="20">
       <c r="A20" t="s">
         <v>43</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="1" t="n">
         <v>1430</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -992,36 +955,36 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="21">
       <c r="A21" t="s">
         <v>49</v>
       </c>
       <c r="B21" s="1"/>
-      <c r="C21" s="1">
+      <c r="C21" s="1" t="n">
         <v>3927</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21" s="1" t="n">
         <v>0.91</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21" s="1" t="n">
         <v>1.52</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="22">
       <c r="A22" t="s">
         <v>50</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="1" t="n">
         <v>585</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -1032,14 +995,14 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="23">
       <c r="A23" t="s">
         <v>50</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="1" t="n">
         <v>3595</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1050,14 +1013,14 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="24">
       <c r="A24" t="s">
         <v>55</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" s="1" t="n">
         <v>1036</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -1068,26 +1031,26 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="25">
       <c r="A25" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="4" t="n">
         <v>3144</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>